<commit_message>
Correggi il link della dashboard e rendi tracciabili i numeri del README
- README: link alla viz Tableau attuale (la v2 non è più pubblicata), origine di
  ogni numero dichiarata, nota sui mesi incompleti e passi di setup del database
- sql/analisi.sql: aggiunte v_kpi_generali, v_retention, v_consegne_recensioni,
  così retention e impatto dei ritardi sono riproducibili dal repository
- notebook/02-ETL: aggiunta la narrazione delle scelte, rimosso il doppio
  caricamento delle tabelle, viste lette da pg_views invece che da un elenco
  scritto a mano, motore Excel esplicito
- result/: anteprima della dashboard aggiornata, export rigenerati, aggiunti
  retention.xlsx e consegne_recensioni.xlsx
- aggiunti data/{raw,processed}/.gitkeep, versioni fissate in requirements.txt,
  licenza MIT versionata
</commit_message>
<xml_diff>
--- a/result/rfm_segmenti.xlsx
+++ b/result/rfm_segmenti.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,86 +441,132 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>pct</t>
+          <t>pct_clienti</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fatturato</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>pct_fatturato</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nel mezzo</t>
+          <t>Campioni</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33332</v>
+        <v>14814</v>
       </c>
       <c r="C2" t="n">
-        <v>34.93</v>
+        <v>15.53</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3979132.06</v>
+      </c>
+      <c r="E2" t="n">
+        <v>29.28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Persi/Basso valore</t>
+          <t>A rischio</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15649</v>
+        <v>14028</v>
       </c>
       <c r="C3" t="n">
-        <v>16.4</v>
+        <v>14.7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3920339.38</v>
+      </c>
+      <c r="E3" t="n">
+        <v>28.84</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Campioni</t>
+          <t>Nel mezzo</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>14937</v>
+        <v>33284</v>
       </c>
       <c r="C4" t="n">
-        <v>15.65</v>
+        <v>34.88</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3721301.46</v>
+      </c>
+      <c r="E4" t="n">
+        <v>27.38</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Nuovi/Promettenti</t>
+          <t>Fedeli (rari)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14740</v>
+        <v>2913</v>
       </c>
       <c r="C5" t="n">
-        <v>15.45</v>
+        <v>3.05</v>
+      </c>
+      <c r="D5" t="n">
+        <v>763291.86</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5.62</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A rischio</t>
+          <t>Persi/Basso valore</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14089</v>
+        <v>15642</v>
       </c>
       <c r="C6" t="n">
-        <v>14.77</v>
+        <v>16.39</v>
+      </c>
+      <c r="D6" t="n">
+        <v>628147.11</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.62</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fedeli (rari)</t>
+          <t>Nuovi/Promettenti</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2673</v>
+        <v>14739</v>
       </c>
       <c r="C7" t="n">
-        <v>2.8</v>
+        <v>15.45</v>
+      </c>
+      <c r="D7" t="n">
+        <v>579431.83</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4.26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>